<commit_message>
Root-domain cleanup: Qatar fashion stores
</commit_message>
<xml_diff>
--- a/markets/fashion/Qatar_Fashion_Stores.xlsx
+++ b/markets/fashion/Qatar_Fashion_Stores.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fashion Stores" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Method" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed - platform subdomain" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7248,7 +7249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7423,7 +7424,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -7433,6 +7433,94 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>Removed 1 rows from Fashion Stores (now 117); each is listed in the Excluded sheet with source "Deliverable cleanup (fashion-stores package)". Website values normalised to clean storefront URLs (5 changed). Counts above (total, type, gender, platform, size tier, verification status) reflect the cleaned list; any by-source/by-channel/signal-origin/QA breakdowns are as at the original run (pre-cleanup).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Root-domain cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rows before</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Kept as-is</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Replaced with root domain</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Removed (no own domain / duplicate of root)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Rows after</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Store Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Old URL</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Reason</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
QA fashion: add 7 StoreLeads gap-fill stores, excluded rows, coverage block, page counts
</commit_message>
<xml_diff>
--- a/markets/fashion/Qatar_Fashion_Stores.xlsx
+++ b/markets/fashion/Qatar_Fashion_Stores.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6905,6 +6905,388 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Luxury Shopping in Qatar</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://51east.com/</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>27603</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Has clothing section</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Women, Men</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>https://51east.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Haneenalsaify</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://www.haneenalsaify.com/</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>767</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>https://www.haneenalsaify.com/products/soft-fit-cotton-hijab</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Lusso Moda</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://lusso-moda.com/</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>537</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>https://lusso-moda.com/products/first-light</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>sheikhastyleboutique</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>https://www.sheikhastyle.com/</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>88</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Wix</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>https://www.sheikhastyle.com/perfumes</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Shop Lamees</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://www.shoplamees.com/</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Not available (sitemap present but yielded no countable URLs; no sitemap/shop total/platform count and no archive captures)</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Salla</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>https://www.shoplamees.com/product/abaya-aneqa-dantel</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ThreeL</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>https://threel.qa/</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>31</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Zid</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>https://threel.qa/products/</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Trendy</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://trendyqatar.com/</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>253</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Ecwid</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>https://trendyqatar.com/products/search</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6916,7 +7298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8742,6 +9124,644 @@
       <c r="D90" t="inlineStr">
         <is>
           <t>Deliverable cleanup (fashion-stores package)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Al Hamim</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://www.alhamim.qa/</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>شركة أمانة لتجارة العسل</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://amanah.qa/</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Blue Lynx Online</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://bluelynxonline.com/</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Dahhas</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://dahhas.com/</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Family Qatar</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://familysupermarket.qa/</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Fnac Qatar</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://fnac.qa/</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>FSAHI</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://fsahi.com/</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Gait</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://gait.com.qa/</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Halaly All You Need</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://www.halalys.com/</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Harmony Organic Matcha Tea</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://www.harmonymatchatea.com/</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>IBN RUSHD PHARMACY</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://www.ibnrushdpharmacy.com/</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>لافيلو تريدنغ</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://la-filo.com/</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>LACOSTE Online Boutique</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://www.lacoste.qa/</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>halafik</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://lakhwiya.com/</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>THE LAST BATCH COFFEE ROASTERS</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://lastbatch.online/</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>LULEA JEWELRY</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://luleajewelryqa.com/</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Maawoon Home Shop</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://maawoon.com/</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>متجر قطر</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://matgarqatar.com/</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Panda Hypermarket</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://panda.qa/</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Qatar Vet Center</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://www.qvcpetshop.com/</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://rarepharmcy.com/</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Reef Perfumes</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://sa.reefperfumes.com/</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>الملكي</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://royalnaturalhoney.com/</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Intertec Group W.L.L.</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://shopintertec.com/</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Silverlow Pharma</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://silverglow.qa/</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Skill Mount Trading</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://skilltechqatar.com/</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>The Football Autograph</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://thefootballautograph.com/</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Voltaat</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://www.voltaat.com/</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>We Sell Everything</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://wse.com.qa/</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
         </is>
       </c>
     </row>
@@ -8756,7 +9776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8783,7 +9803,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>124</t>
         </is>
       </c>
     </row>
@@ -8795,7 +9815,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>{'Fashion-only': 90, 'Has clothing section': 27}</t>
+          <t>{'Fashion-only': 96, 'Has clothing section': 28}</t>
         </is>
       </c>
     </row>
@@ -8807,7 +9827,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>{'Unisex': 61, 'Women': 51, 'Men': 5}</t>
+          <t>{'Unisex': 62, 'Women': 56, 'Men': 5, 'Women, Men': 1}</t>
         </is>
       </c>
     </row>
@@ -9002,89 +10022,100 @@
         <v>117</v>
       </c>
     </row>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Page count</t>
+          <t>StoreLeads gap fill</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rows counted (of 117)</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>98</v>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill of the Qatar directory (see directory workbook, sheet 'Research Coverage')</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Gap stores added to the directory</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Counted by method</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Rows</t>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Gap stores added to the fashion list</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>sitemap</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>86</v>
+          <t>Gap stores not fashion (listed in Excluded)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>archive</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>shop-page total</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-    </row>
+          <t>Fashion rules</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Adult clothing (women, men, unisex) as a fashion-only store or a clothing section; abaya/thobe/modest wear, lingerie and sportswear count; kids-only and shoes/bags/accessories-only do not. Classified from homepage nav/meta and product pages (EN+AR keywords), reviewed manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>sitemap (partial: some child sitemaps unreadable)</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>3</v>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Page count</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>19</v>
-      </c>
-    </row>
+          <t>Rows counted (of 124)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Size distribution (pages per site)</t>
+          <t>Counted by method</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -9096,75 +10127,162 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1-50</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>11</v>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>51-200</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>14</v>
+          <t>archive</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>201-1,000</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>24</v>
+          <t>shop-page total</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1,001-5,000</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>22</v>
+          <t>sitemap (partial: some child sitemaps unreadable)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Size distribution (pages per site)</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1-50</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>51-200</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>201-1,000</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1,001-5,000</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>5,001-20,000</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>20,001-100,000</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>&gt;100,000</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="45" ht="150" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="150" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Method rules: sitemap counted in full (all child sitemaps followed); image and video sitemaps skipped; URLs deduplicated; Arabic and English URLs counted separately; when a sitemap is country-segmented only the listed market's pages are counted; fallbacks, used when no sitemap yields URLs, are the shop-page total, the platform product count (Shopify/WooCommerce) and the web archive (own host only); blocked or unreachable sites are marked Not available and left blank. Child sitemaps that failed are retried up to 4 times (5s/15s/45s/120s); if some still fail the row reads 'sitemap (partial: N of M sitemap files read)' and the count is a lower bound. If the sitemap has country segments but none for the listed market, the whole site is counted when a default storefront exists ('sitemap (whole site, no market segment)', which includes other-country URLs), otherwise the row is Not available.</t>
         </is>
@@ -9172,7 +10290,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A52:C52"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>